<commit_message>
Mejora exportacion de creditos e inventario
</commit_message>
<xml_diff>
--- a/src/lib/server/templates/creditos.xlsx
+++ b/src/lib/server/templates/creditos.xlsx
@@ -1,52 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\angel\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FDA4FAA4-EC08-49C3-814C-CA171E3CD758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B47682D-383A-41DD-A837-2350FF581FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{2D984218-0FA6-4EA0-AAEC-2FA89CD1CB7E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$B$2:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase">Hoja1!$B$2:$J$2</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>FECHA</t>
   </si>
   <si>
+    <t>CLIENTE</t>
+  </si>
+  <si>
+    <t>PRODUCTO</t>
+  </si>
+  <si>
     <t>VALE</t>
   </si>
   <si>
@@ -62,20 +44,22 @@
     <t>DEUDA PENDIENTE</t>
   </si>
   <si>
-    <t>PRODUCTO</t>
-  </si>
-  <si>
-    <t>CLIENTE</t>
+    <t>GALONES</t>
+  </si>
+  <si>
+    <t>REFERENCIA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_-&quot;S/&quot;\ * #,##0.00_-;\-&quot;S/&quot;\ * #,##0.00_-;_-&quot;S/&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -89,6 +73,11 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="3">
@@ -133,10 +122,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -472,45 +473,88 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA81C2F1-6256-472A-864D-3DBF4F728F2E}">
-  <dimension ref="B2:I2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B2:K8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="16.81640625" customWidth="1"/>
-    <col min="6" max="6" width="10.90625" style="3"/>
-    <col min="7" max="7" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.90625" style="3"/>
-    <col min="9" max="9" width="18.7265625" customWidth="1"/>
+    <col min="2" max="2" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.26953125" customWidth="1"/>
+    <col min="5" max="5" width="7.1796875" style="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.90625" style="13" customWidth="1"/>
+    <col min="8" max="8" width="16" style="15" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.90625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="18.7265625" style="15" customWidth="1"/>
+    <col min="11" max="11" width="16.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="2:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>5</v>
-      </c>
+      <c r="K2" s="12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="4"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="I3" s="5"/>
+    </row>
+    <row r="4" spans="2:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="4"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="I4" s="5"/>
+    </row>
+    <row r="5" spans="2:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="4"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="I5" s="5"/>
+    </row>
+    <row r="6" spans="2:11" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="4"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="I6" s="5"/>
+    </row>
+    <row r="8" spans="2:11" s="6" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="14"/>
     </row>
   </sheetData>
-  <autoFilter ref="B2:I2" xr:uid="{EA81C2F1-6256-472A-864D-3DBF4F728F2E}"/>
+  <autoFilter ref="B2:J2" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>